<commit_message>
Actualización de datos Granel Movimientos 2026-10-21 00:56
</commit_message>
<xml_diff>
--- a/Ventas Granel.xlsx
+++ b/Ventas Granel.xlsx
@@ -6688,7 +6688,7 @@
         </is>
       </c>
       <c r="Q98" s="103" t="n">
-        <v>3423608</v>
+        <v>4074094</v>
       </c>
       <c r="R98" s="29" t="n">
         <v>11036</v>
@@ -6736,7 +6736,7 @@
         </is>
       </c>
       <c r="Q99" s="103" t="n">
-        <v>3435620</v>
+        <v>4088388</v>
       </c>
       <c r="R99" s="29" t="n">
         <v>11075</v>
@@ -6796,7 +6796,7 @@
         </is>
       </c>
       <c r="Q100" s="103" t="n">
-        <v>3417602</v>
+        <v>4066946</v>
       </c>
       <c r="R100" s="29" t="n">
         <v>11017</v>

</xml_diff>

<commit_message>
Actualización de datos Granel Movimientos 2026-10-21 01:11
</commit_message>
<xml_diff>
--- a/Ventas Granel.xlsx
+++ b/Ventas Granel.xlsx
@@ -1058,7 +1058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C2:W1024"/>
+  <dimension ref="C2:X1024"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="4.5" customWidth="1" style="81" min="1" max="2"/>
@@ -1186,6 +1186,11 @@
           <t>_Idx_ENAP carga</t>
         </is>
       </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Toneladas Compradas</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="C5" s="7" t="n">
@@ -1249,6 +1254,9 @@
         <f>IF(F5="ENAP carga", COUNTIF(F$5:F5, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X5" t="n">
+        <v>5.93</v>
+      </c>
     </row>
     <row r="6">
       <c r="C6" s="7" t="n">
@@ -2693,6 +2701,9 @@
         <f>IF(F26="ENAP carga", COUNTIF(F$5:F26, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X26" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="C27" s="7" t="n">
@@ -2823,6 +2834,9 @@
         <f>IF(F28="ENAP carga", COUNTIF(F$5:F28, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X28" t="n">
+        <v>5.93</v>
+      </c>
     </row>
     <row r="29">
       <c r="C29" s="7" t="n">
@@ -2963,6 +2977,9 @@
         <f>IF(F30="ENAP carga", COUNTIF(F$5:F30, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X30" t="n">
+        <v>6.02</v>
+      </c>
     </row>
     <row r="31">
       <c r="C31" s="7" t="n">
@@ -3068,6 +3085,9 @@
         <f>IF(F32="ENAP carga", COUNTIF(F$5:F32, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X32" t="n">
+        <v>5.92</v>
+      </c>
     </row>
     <row r="33">
       <c r="C33" s="7" t="n">
@@ -3131,6 +3151,9 @@
         <f>IF(F33="ENAP carga", COUNTIF(F$5:F33, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X33" t="n">
+        <v>5.83</v>
+      </c>
     </row>
     <row r="34">
       <c r="C34" s="7" t="n">
@@ -3656,6 +3679,9 @@
         <f>IF(F41="ENAP carga", COUNTIF(F$5:F41, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X41" t="n">
+        <v>5.83</v>
+      </c>
     </row>
     <row r="42">
       <c r="C42" s="7" t="n">
@@ -3718,6 +3744,9 @@
       <c r="W42">
         <f>IF(F42="ENAP carga", COUNTIF(F$5:F42, "ENAP carga"), "")</f>
         <v/>
+      </c>
+      <c r="X42" t="n">
+        <v>5.52</v>
       </c>
     </row>
     <row r="43">
@@ -3915,6 +3944,9 @@
         <f>IF(F45="ENAP carga", COUNTIF(F$5:F45, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X45" t="n">
+        <v>5.94</v>
+      </c>
     </row>
     <row r="46">
       <c r="C46" s="7" t="n">
@@ -4115,6 +4147,9 @@
         <f>IF(F48="ENAP carga", COUNTIF(F$5:F48, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X48" t="n">
+        <v>5.92</v>
+      </c>
     </row>
     <row r="49" customFormat="1" s="69">
       <c r="C49" s="60" t="n">
@@ -4297,6 +4332,9 @@
       <c r="R51" s="29" t="n">
         <v>11481</v>
       </c>
+      <c r="X51" t="n">
+        <v>5.93</v>
+      </c>
     </row>
     <row r="52">
       <c r="C52" s="7" t="n">
@@ -4502,6 +4540,9 @@
         <f>IF(F54="ENAP carga", COUNTIF(F$5:F54, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X54" t="n">
+        <v>5.83</v>
+      </c>
     </row>
     <row r="55">
       <c r="C55" s="7" t="n">
@@ -4565,6 +4606,9 @@
         <f>IF(F55="ENAP carga", COUNTIF(F$5:F55, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X55" t="n">
+        <v>5.84</v>
+      </c>
     </row>
     <row r="56">
       <c r="C56" s="7" t="n">
@@ -4628,6 +4672,9 @@
         <f>IF(F56="ENAP carga", COUNTIF(F$5:F56, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X56" t="n">
+        <v>5.86</v>
+      </c>
     </row>
     <row r="57">
       <c r="C57" s="7" t="n">
@@ -4691,6 +4738,9 @@
         <f>IF(F57="ENAP carga", COUNTIF(F$5:F57, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X57" t="n">
+        <v>5.83</v>
+      </c>
     </row>
     <row r="58">
       <c r="C58" s="7" t="n">
@@ -4754,6 +4804,9 @@
         <f>IF(F58="ENAP carga", COUNTIF(F$5:F58, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X58" t="n">
+        <v>5.78</v>
+      </c>
     </row>
     <row r="59">
       <c r="C59" s="7" t="n">
@@ -4817,6 +4870,9 @@
         <f>IF(F59="ENAP carga", COUNTIF(F$5:F59, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X59" t="n">
+        <v>5.86</v>
+      </c>
     </row>
     <row r="60">
       <c r="C60" s="7" t="n">
@@ -4880,6 +4936,9 @@
         <f>IF(F60="ENAP carga", COUNTIF(F$5:F60, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X60" t="n">
+        <v>5.78</v>
+      </c>
     </row>
     <row r="61">
       <c r="C61" s="7" t="n">
@@ -4943,6 +5002,9 @@
         <f>IF(F61="ENAP carga", COUNTIF(F$5:F61, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X61" t="n">
+        <v>5.71</v>
+      </c>
     </row>
     <row r="62">
       <c r="C62" s="7" t="n">
@@ -4987,6 +5049,9 @@
       <c r="R62" s="29" t="n">
         <v>11036</v>
       </c>
+      <c r="X62" t="n">
+        <v>5.7</v>
+      </c>
     </row>
     <row r="63">
       <c r="C63" s="7" t="n">
@@ -5031,6 +5096,9 @@
       <c r="R63" s="29" t="n">
         <v>11075</v>
       </c>
+      <c r="X63" t="n">
+        <v>5.72</v>
+      </c>
     </row>
     <row r="64">
       <c r="C64" s="7" t="n">
@@ -5075,6 +5143,9 @@
       <c r="R64" s="29" t="n">
         <v>11055</v>
       </c>
+      <c r="X64" t="n">
+        <v>5.71</v>
+      </c>
     </row>
     <row r="65">
       <c r="C65" s="7" t="n">
@@ -5119,6 +5190,9 @@
       <c r="R65" s="29" t="n">
         <v>11230</v>
       </c>
+      <c r="X65" t="n">
+        <v>5.8</v>
+      </c>
     </row>
     <row r="66">
       <c r="C66" s="7" t="n">
@@ -5163,6 +5237,9 @@
       <c r="R66" s="29" t="n">
         <v>11268</v>
       </c>
+      <c r="X66" t="n">
+        <v>5.82</v>
+      </c>
     </row>
     <row r="67">
       <c r="C67" s="7" t="n">
@@ -5207,6 +5284,9 @@
       <c r="R67" s="29" t="n">
         <v>11094</v>
       </c>
+      <c r="X67" t="n">
+        <v>5.73</v>
+      </c>
     </row>
     <row r="68">
       <c r="C68" s="7" t="n">
@@ -5251,6 +5331,9 @@
       <c r="R68" s="29" t="n">
         <v>11230</v>
       </c>
+      <c r="X68" t="n">
+        <v>5.8</v>
+      </c>
     </row>
     <row r="69">
       <c r="C69" s="7" t="n">
@@ -5295,6 +5378,9 @@
       <c r="R69" s="29" t="n">
         <v>11113</v>
       </c>
+      <c r="X69" t="n">
+        <v>5.74</v>
+      </c>
     </row>
     <row r="70">
       <c r="C70" s="7" t="n">
@@ -5355,6 +5441,9 @@
         <f>IF(F70="ENAP carga", COUNTIF(F$5:F70, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X70" t="n">
+        <v>5.77</v>
+      </c>
     </row>
     <row r="71">
       <c r="C71" s="7" t="n">
@@ -5399,6 +5488,9 @@
       <c r="R71" s="29" t="n">
         <v>11191</v>
       </c>
+      <c r="X71" t="n">
+        <v>5.78</v>
+      </c>
     </row>
     <row r="72">
       <c r="C72" s="7" t="n">
@@ -5442,6 +5534,9 @@
       </c>
       <c r="R72" s="29" t="n">
         <v>11210</v>
+      </c>
+      <c r="X72" t="n">
+        <v>5.79</v>
       </c>
     </row>
     <row r="73">
@@ -5623,6 +5718,9 @@
       <c r="R76" s="29" t="n">
         <v>11172</v>
       </c>
+      <c r="X76" t="n">
+        <v>5.77</v>
+      </c>
     </row>
     <row r="77">
       <c r="C77" s="7" t="n">
@@ -5667,6 +5765,9 @@
       <c r="R77" s="29" t="n">
         <v>11094</v>
       </c>
+      <c r="X77" t="n">
+        <v>5.73</v>
+      </c>
     </row>
     <row r="78">
       <c r="C78" s="7" t="n">
@@ -5711,6 +5812,9 @@
       <c r="R78" s="29" t="n">
         <v>10978</v>
       </c>
+      <c r="X78" t="n">
+        <v>5.67</v>
+      </c>
     </row>
     <row r="79">
       <c r="C79" s="7" t="n">
@@ -5789,6 +5893,9 @@
       <c r="R80" s="29" t="n">
         <v>11210</v>
       </c>
+      <c r="X80" t="n">
+        <v>5.79</v>
+      </c>
     </row>
     <row r="81" customFormat="1" s="79">
       <c r="C81" s="70" t="n">
@@ -5833,6 +5940,9 @@
       <c r="R81" s="78" t="n">
         <v>11172</v>
       </c>
+      <c r="X81" t="n">
+        <v>5.77</v>
+      </c>
     </row>
     <row r="82">
       <c r="C82" s="7" t="n">
@@ -5893,6 +6003,9 @@
         <f>IF(F82="ENAP carga", COUNTIF(F$5:F82, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X82" t="n">
+        <v>5.77</v>
+      </c>
     </row>
     <row r="83">
       <c r="C83" s="7" t="n">
@@ -5937,6 +6050,9 @@
       <c r="R83" s="29" t="n">
         <v>11230</v>
       </c>
+      <c r="X83" t="n">
+        <v>5.8</v>
+      </c>
     </row>
     <row r="84">
       <c r="C84" s="7" t="n">
@@ -5981,6 +6097,9 @@
       <c r="R84" s="29" t="n">
         <v>11191</v>
       </c>
+      <c r="X84" t="n">
+        <v>5.78</v>
+      </c>
     </row>
     <row r="85">
       <c r="C85" s="7" t="n">
@@ -6041,6 +6160,9 @@
         <f>IF(F85="ENAP carga", COUNTIF(F$5:F85, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X85" t="n">
+        <v>5.78</v>
+      </c>
     </row>
     <row r="86">
       <c r="C86" s="7" t="n">
@@ -6085,6 +6207,9 @@
       <c r="R86" s="29" t="n">
         <v>11191</v>
       </c>
+      <c r="X86" t="n">
+        <v>5.78</v>
+      </c>
     </row>
     <row r="87">
       <c r="C87" s="7" t="n">
@@ -6129,6 +6254,9 @@
       <c r="R87" s="29" t="n">
         <v>11055</v>
       </c>
+      <c r="X87" t="n">
+        <v>5.71</v>
+      </c>
     </row>
     <row r="88">
       <c r="C88" s="7" t="n">
@@ -6189,6 +6317,9 @@
         <f>IF(F88="ENAP carga", COUNTIF(F$5:F88, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X88" t="n">
+        <v>5.76</v>
+      </c>
     </row>
     <row r="89">
       <c r="C89" s="7" t="n">
@@ -6233,6 +6364,9 @@
       <c r="R89" s="29" t="n">
         <v>11133</v>
       </c>
+      <c r="X89" t="n">
+        <v>5.75</v>
+      </c>
     </row>
     <row r="90">
       <c r="C90" s="7" t="n">
@@ -6277,6 +6411,9 @@
       <c r="R90" s="29" t="n">
         <v>11133</v>
       </c>
+      <c r="X90" t="n">
+        <v>5.75</v>
+      </c>
     </row>
     <row r="91">
       <c r="C91" s="7" t="n">
@@ -6337,6 +6474,9 @@
         <f>IF(F91="ENAP carga", COUNTIF(F$5:F91, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X91" t="n">
+        <v>5.75</v>
+      </c>
     </row>
     <row r="92">
       <c r="C92" s="7" t="n">
@@ -6381,6 +6521,9 @@
       <c r="R92" s="29" t="n">
         <v>11152</v>
       </c>
+      <c r="X92" t="n">
+        <v>5.76</v>
+      </c>
     </row>
     <row r="93">
       <c r="C93" s="7" t="n">
@@ -6441,6 +6584,9 @@
         <f>IF(F93="ENAP carga", COUNTIF(F$5:F93, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X93" t="n">
+        <v>5.73</v>
+      </c>
     </row>
     <row r="94">
       <c r="C94" s="7" t="n">
@@ -6485,6 +6631,9 @@
       <c r="R94" s="29" t="n">
         <v>11113</v>
       </c>
+      <c r="X94" t="n">
+        <v>5.74</v>
+      </c>
     </row>
     <row r="95">
       <c r="C95" s="7" t="n">
@@ -6545,6 +6694,9 @@
         <f>IF(F95="ENAP carga", COUNTIF(F$5:F95, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X95" t="n">
+        <v>5.76</v>
+      </c>
     </row>
     <row r="96">
       <c r="C96" s="7" t="n">
@@ -6589,6 +6741,9 @@
       <c r="R96" s="29" t="n">
         <v>11113</v>
       </c>
+      <c r="X96" t="n">
+        <v>5.74</v>
+      </c>
     </row>
     <row r="97">
       <c r="C97" s="7" t="n">
@@ -6649,6 +6804,9 @@
         <f>IF(F97="ENAP carga", COUNTIF(F$5:F97, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X97" t="n">
+        <v>5.75</v>
+      </c>
     </row>
     <row r="98">
       <c r="C98" s="7" t="n">
@@ -6697,6 +6855,9 @@
         <f>IF(F98="ENAP carga", COUNTIF(F$5:F98, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X98" t="n">
+        <v>5.7</v>
+      </c>
     </row>
     <row r="99">
       <c r="C99" s="7" t="n">
@@ -6757,6 +6918,9 @@
         <f>IF(F99="ENAP carga", COUNTIF(F$5:F99, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X99" t="n">
+        <v>5.72</v>
+      </c>
     </row>
     <row r="100">
       <c r="C100" s="7" t="n">
@@ -6804,6 +6968,9 @@
       <c r="W100">
         <f>IF(F100="ENAP carga", COUNTIF(F$5:F100, "ENAP carga"), "")</f>
         <v/>
+      </c>
+      <c r="X100" t="n">
+        <v>5.69</v>
       </c>
     </row>
     <row r="101">

</xml_diff>

<commit_message>
Actualización de datos Granel Movimientos 2026-10-22 17:44
</commit_message>
<xml_diff>
--- a/Ventas Granel.xlsx
+++ b/Ventas Granel.xlsx
@@ -4585,7 +4585,7 @@
         </is>
       </c>
       <c r="Q55" s="103" t="n">
-        <v>3675022</v>
+        <v>3713171</v>
       </c>
       <c r="R55" s="29" t="n">
         <v>11307</v>
@@ -6974,10 +6974,24 @@
       </c>
     </row>
     <row r="101">
-      <c r="C101" s="7" t="n"/>
-      <c r="D101" s="1" t="n"/>
-      <c r="E101" s="5" t="n"/>
-      <c r="F101" s="5" t="n"/>
+      <c r="C101" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="D101" s="1" t="inlineStr">
+        <is>
+          <t>ENAP carga</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>VJYL42</t>
+        </is>
+      </c>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>ENAP carga</t>
+        </is>
+      </c>
       <c r="G101" s="1" t="n"/>
       <c r="H101" s="1" t="n"/>
       <c r="I101" s="1" t="n"/>
@@ -6985,11 +6999,23 @@
       <c r="K101" s="38" t="n"/>
       <c r="L101" s="38" t="n"/>
       <c r="M101" s="1" t="n"/>
-      <c r="N101" s="1" t="n"/>
+      <c r="N101" s="1" t="inlineStr">
+        <is>
+          <t>ENAP carga</t>
+        </is>
+      </c>
       <c r="O101" s="102" t="n"/>
-      <c r="P101" s="26" t="n"/>
-      <c r="Q101" s="103" t="n"/>
-      <c r="R101" s="29" t="n"/>
+      <c r="P101" s="26" t="inlineStr">
+        <is>
+          <t>Guía N° 2378891</t>
+        </is>
+      </c>
+      <c r="Q101" s="103" t="n">
+        <v>4095536</v>
+      </c>
+      <c r="R101" s="29" t="n">
+        <v>11094</v>
+      </c>
       <c r="T101">
         <f>IF(F101="CJ", COUNTIF(F$5:F101, "CJ"), "")</f>
         <v/>
@@ -7006,12 +7032,29 @@
         <f>IF(F101="ENAP carga", COUNTIF(F$5:F101, "ENAP carga"), "")</f>
         <v/>
       </c>
+      <c r="X101" t="n">
+        <v>5.73</v>
+      </c>
     </row>
     <row r="102">
-      <c r="C102" s="7" t="n"/>
-      <c r="D102" s="1" t="n"/>
-      <c r="E102" s="5" t="n"/>
-      <c r="F102" s="5" t="n"/>
+      <c r="C102" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="D102" s="1" t="inlineStr">
+        <is>
+          <t>ENAP carga</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>VJYL61</t>
+        </is>
+      </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>ENAP carga</t>
+        </is>
+      </c>
       <c r="G102" s="1" t="n"/>
       <c r="H102" s="101" t="n"/>
       <c r="I102" s="5" t="n"/>
@@ -7019,11 +7062,30 @@
       <c r="K102" s="34" t="n"/>
       <c r="L102" s="34" t="n"/>
       <c r="M102" s="102" t="n"/>
-      <c r="N102" s="1" t="n"/>
+      <c r="N102" s="1" t="inlineStr">
+        <is>
+          <t>ENAP carga</t>
+        </is>
+      </c>
       <c r="O102" s="102" t="n"/>
-      <c r="P102" s="26" t="n"/>
-      <c r="Q102" s="103" t="n"/>
-      <c r="R102" s="29" t="n"/>
+      <c r="P102" s="26" t="inlineStr">
+        <is>
+          <t>Guía N° 2378923</t>
+        </is>
+      </c>
+      <c r="Q102" s="103" t="n">
+        <v>4088388</v>
+      </c>
+      <c r="R102" s="29" t="n">
+        <v>11075</v>
+      </c>
+      <c r="W102">
+        <f>IF(F102="ENAP carga", COUNTIF(F$5:F102, "ENAP carga"), "")</f>
+        <v/>
+      </c>
+      <c r="X102" t="n">
+        <v>5.72</v>
+      </c>
     </row>
     <row r="103">
       <c r="C103" s="7" t="n"/>

</xml_diff>